<commit_message>
Update Evaluation Form and Eval Documentation
</commit_message>
<xml_diff>
--- a/docs/assets/Capstone-Project-Final-Evaluation.xlsx
+++ b/docs/assets/Capstone-Project-Final-Evaluation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10526"/>
   <workbookPr showInkAnnotation="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ernesto/github/MHACapstone/docs/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F415B934-E26A-3041-A5D1-C81A526ED69D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94EE1698-6AD9-A44B-BDF8-CDF9D6F12712}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25660" yWindow="660" windowWidth="25380" windowHeight="27980" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="56040" yWindow="4120" windowWidth="25360" windowHeight="18880" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="OVERALL GRADE" sheetId="3" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Chair Evaluation" sheetId="4" r:id="rId3"/>
     <sheet name="Mentor Evaluation" sheetId="2" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateCount="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr defaultImageDpi="32767"/>
@@ -303,7 +303,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="119">
   <si>
     <t>Final Capstone Project Evaluation Form</t>
   </si>
@@ -446,18 +446,6 @@
     <t>Capstone Report and Presentation Score Sheet</t>
   </si>
   <si>
-    <t xml:space="preserve">Use this form to evaluate the written Capstone Report and Poster Presentation. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Note: Please refer to the linked rubrics and guidelines (links underlined below) for your evaluation. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Note: this portion of the evaluation represents 85% of the final grade </t>
-  </si>
-  <si>
-    <t>Part 1 - Written Report (guidelines) - 70%</t>
-  </si>
-  <si>
     <t>Written Report Grading Rubric</t>
   </si>
   <si>
@@ -518,22 +506,7 @@
     <t>Converted Percentage</t>
   </si>
   <si>
-    <t>Part 2 - Poster Presentation (guidelines) - 30%</t>
-  </si>
-  <si>
     <t>Poster Grading Rubric</t>
-  </si>
-  <si>
-    <t>Poster Composition and grammar</t>
-  </si>
-  <si>
-    <t>Poster Figures and Images</t>
-  </si>
-  <si>
-    <t>Poster Presentation: Presence</t>
-  </si>
-  <si>
-    <t>Poster Presentation: Questions</t>
   </si>
   <si>
     <t>Overall Percentage for Report and Presentation</t>
@@ -590,15 +563,6 @@
     <t xml:space="preserve">... was able to work independently. </t>
   </si>
   <si>
-    <t xml:space="preserve">... set and met internal deadlines to keep his/her project on task. </t>
-  </si>
-  <si>
-    <t>... met final deadlines imposed by the MHA program for submitting forms, printing poster and turning in the Final Report.</t>
-  </si>
-  <si>
-    <t>... was professional and punctual in face-to-face meetings with committee members.</t>
-  </si>
-  <si>
     <t>... was professional and punctual in email exchanges with committee members.</t>
   </si>
   <si>
@@ -656,9 +620,6 @@
     <t>For the evaluation of the MHA Capstone project (by the Capstone Committee)</t>
   </si>
   <si>
-    <t>Revised: 01/24/2025</t>
-  </si>
-  <si>
     <t>Range: 0-10</t>
   </si>
   <si>
@@ -681,6 +642,45 @@
   </si>
   <si>
     <t>Great, Minor Revisions</t>
+  </si>
+  <si>
+    <t>Background Hypothesis/Objective</t>
+  </si>
+  <si>
+    <t>Conclusions and Future Work</t>
+  </si>
+  <si>
+    <t>Poster Design and Aesthetics</t>
+  </si>
+  <si>
+    <t>Stage Presence</t>
+  </si>
+  <si>
+    <t>Answering Questions</t>
+  </si>
+  <si>
+    <t>... was professional and punctual in meetings and communications.</t>
+  </si>
+  <si>
+    <t>... Asked questions and kept diligent notes.</t>
+  </si>
+  <si>
+    <t>... exhibited progressive improvement and academic growth, culminating in a master of the capstone topic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">... set and met internal deadlines to keep the project on task. </t>
+  </si>
+  <si>
+    <t>Part 1 - Written Report (guidelines)</t>
+  </si>
+  <si>
+    <t>Part 2 - Poster Presentation (guidelines)</t>
+  </si>
+  <si>
+    <t>To evaluate the written Capstone Report and Poster Presentation</t>
+  </si>
+  <si>
+    <t>Revised: 06/10/2025</t>
   </si>
 </sst>
 </file>
@@ -691,7 +691,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="35" x14ac:knownFonts="1">
+  <fonts count="37" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -948,6 +948,21 @@
       <name val="Tw Cen MT Condensed"/>
       <family val="2"/>
       <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Tw Cen MT"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="0" tint="-0.499984740745262"/>
+      <name val="Tw Cen MT"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="13">
@@ -1197,7 +1212,7 @@
     <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="19" fillId="8" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1358,6 +1373,16 @@
     <xf numFmtId="49" fontId="8" fillId="12" borderId="3" xfId="18" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="8" fillId="12" borderId="6" xfId="18" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="7" fillId="10" borderId="9" xfId="24" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="25">
     <cellStyle name="Accent1" xfId="6" builtinId="29"/>
@@ -1474,14 +1499,15 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>84666</xdr:colOff>
+      <xdr:colOff>143933</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>8466</xdr:rowOff>
+      <xdr:rowOff>50798</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4495800" cy="4080933"/>
+    <xdr:ext cx="4495800" cy="4097867"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="2" name="TextBox 1">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
@@ -1492,8 +1518,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5477933" y="1159933"/>
-          <a:ext cx="4495800" cy="4080933"/>
+          <a:off x="5537200" y="1202265"/>
+          <a:ext cx="4495800" cy="4097867"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1699,7 +1725,17 @@
           <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
         </a:p>
         <a:p>
-          <a:endParaRPr lang="en-US" sz="1100"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t>Be sure to refer to the Capstone Evalution Documentation and posted Rubrics as you evaluate their assignments: </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US">
+              <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id=""/>
+            </a:rPr>
+            <a:t>Final Evaluation - Modern Human Anatomy Capstone Project</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -1716,7 +1752,7 @@
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Score"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Total Possible"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Missing Data" dataDxfId="9">
-      <calculatedColumnFormula>COUNTBLANK('Report and Presentation'!C12:E18) + COUNTBLANK('Report and Presentation'!C25:E26)</calculatedColumnFormula>
+      <calculatedColumnFormula>COUNTBLANK('Report and Presentation'!C7:E13) + COUNTBLANK('Report and Presentation'!C20:E24)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1726,6 +1762,9 @@
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table3" displayName="Table3" ref="A24:C36" totalsRowShown="0" headerRowDxfId="8">
   <autoFilter ref="A24:C36" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A25:C36">
+    <sortCondition descending="1" ref="B24:B36"/>
+  </sortState>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Letter grade"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Percentage"/>
@@ -1736,10 +1775,10 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table2" displayName="Table2" ref="G8:I19" totalsRowShown="0" dataDxfId="7" headerRowCellStyle="Accent1">
-  <autoFilter ref="G8:I19" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G7:G15">
-    <sortCondition ref="G6:G15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table2" displayName="Table2" ref="G3:I14" totalsRowShown="0" dataDxfId="7" headerRowCellStyle="Accent1">
+  <autoFilter ref="G3:I14" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G4:I14">
+    <sortCondition descending="1" ref="G3:G14"/>
   </sortState>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Score" dataDxfId="6"/>
@@ -1762,8 +1801,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table4" displayName="Table4" ref="A11:B26" totalsRowShown="0" headerRowCellStyle="Accent1">
-  <autoFilter ref="A11:B26" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table4" displayName="Table4" ref="A11:B24" totalsRowShown="0" headerRowCellStyle="Accent1">
+  <autoFilter ref="A11:B24" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="2">
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="The Student…" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Score_x000a_Range: 0-1" dataDxfId="0"/>
@@ -2062,12 +2101,12 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="48" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -2099,7 +2138,7 @@
       </c>
       <c r="B8" s="50"/>
       <c r="C8" s="11" t="e">
-        <f>'Report and Presentation'!C33</f>
+        <f>'Report and Presentation'!C31</f>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -2109,7 +2148,7 @@
       </c>
       <c r="B9" s="50"/>
       <c r="C9" s="11" t="e">
-        <f>'Report and Presentation'!D33</f>
+        <f>'Report and Presentation'!D31</f>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -2119,7 +2158,7 @@
       </c>
       <c r="B10" s="50"/>
       <c r="C10" s="11" t="e">
-        <f>'Report and Presentation'!E33</f>
+        <f>'Report and Presentation'!E31</f>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -2143,15 +2182,15 @@
         <v>12</v>
       </c>
       <c r="B13" s="9" t="e">
-        <f>Table1[[#This Row],[Total Possible]]*'Report and Presentation'!C34</f>
+        <f>Table1[[#This Row],[Total Possible]]*'Report and Presentation'!C32</f>
         <v>#DIV/0!</v>
       </c>
       <c r="C13">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="D13" s="6">
-        <f>COUNTBLANK('Report and Presentation'!C12:E18) + COUNTBLANK('Report and Presentation'!C25:E26)</f>
-        <v>27</v>
+        <f>COUNTBLANK('Report and Presentation'!C7:E13) + COUNTBLANK('Report and Presentation'!C20:E24)</f>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
@@ -2159,20 +2198,20 @@
         <v>13</v>
       </c>
       <c r="B14" s="9" t="e">
-        <f>'Mentor Evaluation'!B26</f>
+        <f>'Mentor Evaluation'!B24</f>
         <v>#DIV/0!</v>
       </c>
       <c r="C14">
         <v>5</v>
       </c>
       <c r="D14" s="6">
-        <f>COUNTBLANK('Mentor Evaluation'!B12:B24)</f>
-        <v>13</v>
+        <f>COUNTBLANK('Mentor Evaluation'!B12:B22)</f>
+        <v>11</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="52" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="B15" s="9" t="e">
         <f>'Chair Evaluation'!B23</f>
@@ -2188,11 +2227,11 @@
     </row>
     <row r="16" spans="1:4" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="B16" s="53"/>
       <c r="C16">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D16" s="6"/>
     </row>
@@ -2221,7 +2260,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
@@ -2246,135 +2285,135 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="36" t="s">
-        <v>21</v>
-      </c>
-      <c r="B25" s="36" t="s">
-        <v>22</v>
-      </c>
-      <c r="C25" s="36">
-        <v>0</v>
+      <c r="A25" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="B25" s="38" t="s">
+        <v>44</v>
+      </c>
+      <c r="C25" s="38">
+        <v>93</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="36" t="s">
-        <v>23</v>
-      </c>
-      <c r="B26" s="36" t="s">
-        <v>24</v>
-      </c>
-      <c r="C26" s="36">
-        <v>60</v>
+      <c r="A26" s="38" t="s">
+        <v>41</v>
+      </c>
+      <c r="B26" s="38" t="s">
+        <v>42</v>
+      </c>
+      <c r="C26" s="38">
+        <v>90</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="36" t="s">
-        <v>25</v>
-      </c>
-      <c r="B27" s="36" t="s">
-        <v>26</v>
-      </c>
-      <c r="C27" s="36">
-        <v>63</v>
+      <c r="A27" s="37" t="s">
+        <v>39</v>
+      </c>
+      <c r="B27" s="37" t="s">
+        <v>40</v>
+      </c>
+      <c r="C27" s="37">
+        <v>87</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="B28" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="C28" s="36">
-        <v>67</v>
+      <c r="A28" s="37" t="s">
+        <v>37</v>
+      </c>
+      <c r="B28" s="37" t="s">
+        <v>38</v>
+      </c>
+      <c r="C28" s="37">
+        <v>83</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="36" t="s">
-        <v>29</v>
-      </c>
-      <c r="B29" s="36" t="s">
-        <v>30</v>
-      </c>
-      <c r="C29" s="36">
-        <v>70</v>
+      <c r="A29" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="B29" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="C29" s="37">
+        <v>80</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="36" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B30" s="36" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C30" s="36">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="36" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B31" s="36" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C31" s="36">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="37" t="s">
-        <v>35</v>
-      </c>
-      <c r="B32" s="37" t="s">
-        <v>36</v>
-      </c>
-      <c r="C32" s="37">
-        <v>80</v>
+      <c r="A32" s="36" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="C32" s="36">
+        <v>70</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" s="37" t="s">
-        <v>37</v>
-      </c>
-      <c r="B33" s="37" t="s">
-        <v>38</v>
-      </c>
-      <c r="C33" s="37">
-        <v>83</v>
+      <c r="A33" s="36" t="s">
+        <v>27</v>
+      </c>
+      <c r="B33" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="C33" s="36">
+        <v>67</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A34" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="B34" s="37" t="s">
-        <v>40</v>
-      </c>
-      <c r="C34" s="37">
-        <v>87</v>
+      <c r="A34" s="36" t="s">
+        <v>25</v>
+      </c>
+      <c r="B34" s="36" t="s">
+        <v>26</v>
+      </c>
+      <c r="C34" s="36">
+        <v>63</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35" s="38" t="s">
-        <v>41</v>
-      </c>
-      <c r="B35" s="38" t="s">
-        <v>42</v>
-      </c>
-      <c r="C35" s="38">
-        <v>90</v>
+      <c r="A35" s="36" t="s">
+        <v>23</v>
+      </c>
+      <c r="B35" s="36" t="s">
+        <v>24</v>
+      </c>
+      <c r="C35" s="36">
+        <v>60</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A36" s="38" t="s">
-        <v>43</v>
-      </c>
-      <c r="B36" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="C36" s="38">
-        <v>93</v>
+      <c r="A36" s="36" t="s">
+        <v>21</v>
+      </c>
+      <c r="B36" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="C36" s="36">
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
@@ -2383,7 +2422,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" selectLockedCells="1"/>
+  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A26:C37">
     <sortCondition ref="C12"/>
   </sortState>
@@ -2432,7 +2471,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.42578125" customWidth="1"/>
@@ -2446,487 +2485,503 @@
     <col min="9" max="9" width="27.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="23" x14ac:dyDescent="0.25">
-      <c r="A1" s="75" t="s">
+    <row r="1" spans="1:9" ht="31" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="81" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="1"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="I3" s="44"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" s="2"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6" s="5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" s="2" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="61"/>
-      <c r="B8" s="62" t="s">
-        <v>50</v>
-      </c>
-      <c r="C8" s="63" t="str">
+    </row>
+    <row r="2" spans="1:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="82" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" s="2" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="61"/>
+      <c r="B3" s="62" t="s">
+        <v>115</v>
+      </c>
+      <c r="C3" s="63" t="str">
         <f>'OVERALL GRADE'!A8</f>
         <v>Mentor</v>
       </c>
-      <c r="D8" s="63" t="str">
+      <c r="D3" s="63" t="str">
         <f>'OVERALL GRADE'!A9</f>
         <v>Member 1</v>
       </c>
-      <c r="E8" s="63" t="str">
+      <c r="E3" s="63" t="str">
         <f>'OVERALL GRADE'!A10</f>
         <v>Member 2</v>
       </c>
-      <c r="F8"/>
-      <c r="G8" s="25" t="s">
+      <c r="F3"/>
+      <c r="G3" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="H8" s="55" t="s">
-        <v>117</v>
-      </c>
-      <c r="I8" s="25" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="60" t="s">
+      <c r="H3" s="55" t="s">
+        <v>104</v>
+      </c>
+      <c r="I3" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="7">
+    </row>
+    <row r="4" spans="1:9" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="B4" s="60" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="7">
         <f>'OVERALL GRADE'!B8</f>
         <v>0</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D4" s="7">
         <f>'OVERALL GRADE'!B9</f>
         <v>0</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E4" s="7">
         <f>'OVERALL GRADE'!B10</f>
         <v>0</v>
       </c>
-      <c r="G9" s="33">
-        <v>0</v>
-      </c>
-      <c r="H9" s="56" t="s">
-        <v>21</v>
-      </c>
-      <c r="I9" s="30" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="19" x14ac:dyDescent="0.2">
-      <c r="C10" s="73" t="s">
+      <c r="G4" s="35">
+        <v>10</v>
+      </c>
+      <c r="H4" s="58" t="s">
+        <v>43</v>
+      </c>
+      <c r="I4" s="32" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="19" x14ac:dyDescent="0.2">
+      <c r="C5" s="73" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" s="73" t="s">
+        <v>49</v>
+      </c>
+      <c r="E5" s="73" t="s">
+        <v>50</v>
+      </c>
+      <c r="G5" s="35">
+        <v>9.5</v>
+      </c>
+      <c r="H5" s="58" t="s">
+        <v>43</v>
+      </c>
+      <c r="I5" s="32" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" s="2" customFormat="1" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="65"/>
+      <c r="B6" s="74" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="F6"/>
+      <c r="G6" s="35">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="H6" s="58" t="s">
+        <v>43</v>
+      </c>
+      <c r="I6" s="32" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="66" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="67" t="s">
         <v>52</v>
       </c>
-      <c r="D10" s="73" t="s">
-        <v>53</v>
-      </c>
-      <c r="E10" s="73" t="s">
+      <c r="C7" s="46"/>
+      <c r="D7" s="46"/>
+      <c r="E7" s="46"/>
+      <c r="G7" s="35">
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="H7" s="58" t="s">
+        <v>41</v>
+      </c>
+      <c r="I7" s="45"/>
+    </row>
+    <row r="8" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" t="s">
         <v>54</v>
       </c>
-      <c r="G10" s="33">
-        <v>7.9</v>
-      </c>
-      <c r="H10" s="56" t="s">
-        <v>33</v>
-      </c>
-      <c r="I10" s="30" t="s">
+      <c r="C8" s="46"/>
+      <c r="D8" s="46"/>
+      <c r="E8" s="46"/>
+      <c r="G8" s="35">
+        <v>9</v>
+      </c>
+      <c r="H8" s="58" t="s">
+        <v>41</v>
+      </c>
+      <c r="I8" s="32" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" s="46"/>
+      <c r="D9" s="46"/>
+      <c r="E9" s="46"/>
+      <c r="G9" s="34">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="H9" s="57" t="s">
+        <v>39</v>
+      </c>
+      <c r="I9" s="31" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="46"/>
+      <c r="D10" s="46"/>
+      <c r="E10" s="46"/>
+      <c r="G10" s="34">
+        <v>8.5</v>
+      </c>
+      <c r="H10" s="57" t="s">
+        <v>37</v>
+      </c>
+      <c r="I10" s="31" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" s="2" customFormat="1" ht="20" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="65"/>
-      <c r="B11" s="74" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="D11" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="E11" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="F11"/>
+      <c r="B11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" s="46"/>
+      <c r="D11" s="46"/>
+      <c r="E11" s="46"/>
       <c r="G11" s="34">
-        <v>8</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="H11" s="57" t="s">
         <v>35</v>
       </c>
       <c r="I11" s="31" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" t="s">
         <v>61</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="66" t="s">
-        <v>43</v>
-      </c>
-      <c r="B12" s="67" t="s">
-        <v>56</v>
       </c>
       <c r="C12" s="46"/>
       <c r="D12" s="46"/>
       <c r="E12" s="46"/>
       <c r="G12" s="34">
-        <v>8.1999999999999993</v>
+        <v>8</v>
       </c>
       <c r="H12" s="57" t="s">
         <v>35</v>
       </c>
       <c r="I12" s="31" t="s">
-        <v>112</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="B13" t="s">
-        <v>58</v>
+      <c r="A13" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>63</v>
       </c>
       <c r="C13" s="46"/>
       <c r="D13" s="46"/>
       <c r="E13" s="46"/>
-      <c r="G13" s="34">
-        <v>8.5</v>
-      </c>
-      <c r="H13" s="57" t="s">
-        <v>37</v>
-      </c>
-      <c r="I13" s="31" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="B14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C14" s="46"/>
-      <c r="D14" s="46"/>
-      <c r="E14" s="46"/>
-      <c r="G14" s="34">
-        <v>8.6999999999999993</v>
-      </c>
-      <c r="H14" s="57" t="s">
-        <v>39</v>
-      </c>
-      <c r="I14" s="31" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="B15" t="s">
-        <v>62</v>
-      </c>
-      <c r="C15" s="46"/>
-      <c r="D15" s="46"/>
-      <c r="E15" s="46"/>
-      <c r="G15" s="35">
-        <v>9</v>
-      </c>
-      <c r="H15" s="58" t="s">
-        <v>41</v>
-      </c>
-      <c r="I15" s="32" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="B16" t="s">
-        <v>64</v>
-      </c>
-      <c r="C16" s="46"/>
-      <c r="D16" s="46"/>
-      <c r="E16" s="46"/>
-      <c r="G16" s="35">
-        <v>9.1999999999999993</v>
-      </c>
-      <c r="H16" s="58" t="s">
-        <v>41</v>
-      </c>
-      <c r="I16" s="45"/>
-    </row>
-    <row r="17" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
+      <c r="G13" s="33">
+        <v>7.9</v>
+      </c>
+      <c r="H13" s="56" t="s">
+        <v>33</v>
+      </c>
+      <c r="I13" s="30" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="17"/>
+      <c r="B14" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" s="28" t="e">
+        <f>AVERAGE(C7:C13)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D14" s="27" t="e">
+        <f>AVERAGE(D7:D13)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E14" s="27" t="e">
+        <f>AVERAGE(E7:E13)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G14" s="33">
+        <v>0</v>
+      </c>
+      <c r="H14" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="B17" t="s">
-        <v>65</v>
-      </c>
-      <c r="C17" s="46"/>
-      <c r="D17" s="46"/>
-      <c r="E17" s="46"/>
-      <c r="G17" s="35">
-        <v>9.3000000000000007</v>
-      </c>
-      <c r="H17" s="58" t="s">
-        <v>43</v>
-      </c>
-      <c r="I17" s="32" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="15" t="s">
+      <c r="I14" s="30" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" s="17"/>
+      <c r="B15" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="B18" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="C18" s="46"/>
-      <c r="D18" s="46"/>
-      <c r="E18" s="46"/>
-      <c r="G18" s="35">
-        <v>9.5</v>
-      </c>
-      <c r="H18" s="58" t="s">
-        <v>43</v>
-      </c>
-      <c r="I18" s="32" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="17"/>
-      <c r="B19" s="18" t="s">
-        <v>69</v>
-      </c>
-      <c r="C19" s="28" t="e">
-        <f>AVERAGE(C12:C18)</f>
+      <c r="C15" s="26" t="e">
+        <f>C14/10</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D19" s="27" t="e">
-        <f>AVERAGE(D12:D18)</f>
+      <c r="D15" s="26" t="e">
+        <f t="shared" ref="D15:E15" si="0">D14/10</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E19" s="27" t="e">
-        <f>AVERAGE(E12:E18)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G19" s="35">
-        <v>10</v>
-      </c>
-      <c r="H19" s="58" t="s">
-        <v>43</v>
-      </c>
-      <c r="I19" s="32" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A20" s="17"/>
-      <c r="B20" s="18" t="s">
-        <v>70</v>
-      </c>
-      <c r="C20" s="26" t="e">
-        <f>C19/10</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D20" s="26" t="e">
-        <f t="shared" ref="D20:E20" si="0">D19/10</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E20" s="26" t="e">
+      <c r="E15" s="26" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="22" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="61"/>
-      <c r="B22" s="64" t="s">
-        <v>71</v>
-      </c>
-      <c r="C22" s="61"/>
-      <c r="D22" s="61"/>
-      <c r="E22" s="61"/>
-      <c r="F22"/>
-      <c r="H22" s="59"/>
-    </row>
-    <row r="23" spans="1:9" s="2" customFormat="1" ht="19" x14ac:dyDescent="0.2">
-      <c r="A23" s="22"/>
-      <c r="B23" s="60" t="s">
-        <v>72</v>
-      </c>
-      <c r="C23" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="D23" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="E23" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="F23"/>
-      <c r="G23"/>
-      <c r="H23" s="54"/>
-      <c r="I23" s="24"/>
-    </row>
-    <row r="24" spans="1:9" ht="20" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="65"/>
-      <c r="B24" s="74" t="s">
+    <row r="17" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="61"/>
+      <c r="B17" s="64" t="s">
+        <v>116</v>
+      </c>
+      <c r="C17" s="61"/>
+      <c r="D17" s="61"/>
+      <c r="E17" s="61"/>
+      <c r="F17"/>
+      <c r="H17" s="59"/>
+    </row>
+    <row r="18" spans="1:9" s="2" customFormat="1" ht="19" x14ac:dyDescent="0.2">
+      <c r="A18" s="22"/>
+      <c r="B18" s="60" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="D18" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="E18" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="F18"/>
+      <c r="G18"/>
+      <c r="H18" s="54"/>
+      <c r="I18" s="24"/>
+    </row>
+    <row r="19" spans="1:9" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="65"/>
+      <c r="B19" s="74" t="s">
         <v>8</v>
       </c>
-      <c r="C24" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="D24" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="E24" s="21" t="s">
-        <v>111</v>
-      </c>
+      <c r="C19" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="D19" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="E19" s="21" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="68" t="s">
+        <v>43</v>
+      </c>
+      <c r="B20" s="67" t="s">
+        <v>106</v>
+      </c>
+      <c r="C20" s="46"/>
+      <c r="D20" s="46"/>
+      <c r="E20" s="46"/>
+    </row>
+    <row r="21" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="69" t="s">
+        <v>37</v>
+      </c>
+      <c r="B21" s="43" t="s">
+        <v>56</v>
+      </c>
+      <c r="C21" s="46"/>
+      <c r="D21" s="46"/>
+      <c r="E21" s="46"/>
+    </row>
+    <row r="22" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="69" t="s">
+        <v>31</v>
+      </c>
+      <c r="B22" s="43" t="s">
+        <v>58</v>
+      </c>
+      <c r="C22" s="46"/>
+      <c r="D22" s="46"/>
+      <c r="E22" s="46"/>
+    </row>
+    <row r="23" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="69" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="43" t="s">
+        <v>107</v>
+      </c>
+      <c r="C23" s="46"/>
+      <c r="D23" s="46"/>
+      <c r="E23" s="46"/>
+    </row>
+    <row r="24" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="69" t="s">
+        <v>59</v>
+      </c>
+      <c r="B24" s="43" t="s">
+        <v>108</v>
+      </c>
+      <c r="C24" s="46"/>
+      <c r="D24" s="46"/>
+      <c r="E24" s="46"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="59"/>
+      <c r="I24" s="2"/>
     </row>
     <row r="25" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="68" t="s">
-        <v>43</v>
-      </c>
-      <c r="B25" s="67" t="s">
-        <v>73</v>
+      <c r="A25" s="69" t="s">
+        <v>21</v>
+      </c>
+      <c r="B25" s="43" t="s">
+        <v>109</v>
       </c>
       <c r="C25" s="46"/>
       <c r="D25" s="46"/>
       <c r="E25" s="46"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="59"/>
+      <c r="I25" s="44"/>
     </row>
     <row r="26" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="69" t="s">
-        <v>37</v>
-      </c>
-      <c r="B26" s="43" t="s">
-        <v>74</v>
+      <c r="A26" s="70" t="s">
+        <v>62</v>
+      </c>
+      <c r="B26" s="71" t="s">
+        <v>110</v>
       </c>
       <c r="C26" s="46"/>
       <c r="D26" s="46"/>
       <c r="E26" s="46"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="59"/>
-      <c r="I26" s="2"/>
-    </row>
-    <row r="27" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="69" t="s">
-        <v>31</v>
-      </c>
-      <c r="B27" s="43" t="s">
-        <v>75</v>
-      </c>
-      <c r="C27" s="46"/>
-      <c r="D27" s="46"/>
-      <c r="E27" s="46"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="59"/>
-      <c r="I27" s="44"/>
-    </row>
-    <row r="28" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="70" t="s">
-        <v>25</v>
-      </c>
-      <c r="B28" s="71" t="s">
-        <v>76</v>
-      </c>
-      <c r="C28" s="46"/>
-      <c r="D28" s="46"/>
-      <c r="E28" s="46"/>
-    </row>
-    <row r="29" spans="1:9" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="17"/>
-      <c r="B29" s="18" t="s">
-        <v>69</v>
-      </c>
-      <c r="C29" s="9" t="e">
-        <f t="shared" ref="C29:E29" si="1">AVERAGE(C25:C28)</f>
+    </row>
+    <row r="27" spans="1:9" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="17"/>
+      <c r="B27" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="C27" s="9" t="e">
+        <f t="shared" ref="C27:E27" si="1">AVERAGE(C20:C26)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D29" s="9" t="e">
+      <c r="D27" s="9" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="E29" s="9" t="e">
+      <c r="E27" s="9" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B30" s="18" t="s">
-        <v>70</v>
-      </c>
-      <c r="C30" s="26" t="e">
-        <f>C29/10</f>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B28" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="C28" s="26" t="e">
+        <f>C27/10</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D30" s="26" t="e">
-        <f t="shared" ref="D30:E30" si="2">D29/10</f>
+      <c r="D28" s="26" t="e">
+        <f t="shared" ref="D28:E28" si="2">D27/10</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E30" s="26" t="e">
+      <c r="E28" s="26" t="e">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A32" s="61"/>
-      <c r="B32" s="61" t="s">
-        <v>77</v>
-      </c>
-      <c r="C32" s="61"/>
-      <c r="D32" s="61"/>
-      <c r="E32" s="61"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B33" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C33" s="19" t="e">
-        <f>(C19*0.7 +C29* 0.3)/10</f>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A30" s="61"/>
+      <c r="B30" s="61" t="s">
+        <v>68</v>
+      </c>
+      <c r="C30" s="61"/>
+      <c r="D30" s="61"/>
+      <c r="E30" s="61"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B31" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C31" s="19" t="e">
+        <f>(C14*0.5 +C27* 0.5)/10</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D33" s="19" t="e">
-        <f t="shared" ref="D33:E33" si="3">(D19*0.7 +D29* 0.3)/10</f>
+      <c r="D31" s="19" t="e">
+        <f t="shared" ref="D31:E31" si="3">(D14*0.7 +D27* 0.3)/10</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E33" s="19" t="e">
+      <c r="E31" s="19" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A34" s="29"/>
-      <c r="B34" s="72" t="s">
-        <v>79</v>
-      </c>
-      <c r="C34" s="13" t="e">
-        <f>AVERAGE(C33:E33)</f>
+    <row r="32" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A32" s="29"/>
+      <c r="B32" s="72" t="s">
+        <v>70</v>
+      </c>
+      <c r="C32" s="13" t="e">
+        <f>AVERAGE(C31:E31)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D34" s="10"/>
-      <c r="E34" s="10"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1"/>
+  <sheetProtection sheet="1" selectLockedCells="1"/>
   <phoneticPr fontId="9" type="noConversion"/>
-  <conditionalFormatting sqref="C29:E29">
+  <conditionalFormatting sqref="C27:E27">
     <cfRule type="colorScale" priority="13">
       <colorScale>
         <cfvo type="num" val="7.9"/>
@@ -2938,7 +2993,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C33:E33 C34">
+  <conditionalFormatting sqref="C31:E31 C32">
     <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="num" val="0.75"/>
@@ -2950,7 +3005,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C19:F19">
+  <conditionalFormatting sqref="C14:F14">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="num" val="7.9"/>
@@ -2962,7 +3017,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C20:F20 C30:E30">
+  <conditionalFormatting sqref="C15:F15 C28:E28">
     <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="num" val="0.79"/>
@@ -2975,20 +3030,20 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="decimal" errorStyle="information" allowBlank="1" showErrorMessage="1" errorTitle="Out of range" error="Enter value between 1 and 5" promptTitle="Score Range" prompt="Between 1 and 5" sqref="C12:E18" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="decimal" errorStyle="information" allowBlank="1" showErrorMessage="1" errorTitle="Out of range" error="Enter value between 1 and 5" promptTitle="Score Range" prompt="Between 1 and 5" sqref="C7:E13" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>0</formula1>
       <formula2>10</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="Range error" error="Value not between 1 and 5" promptTitle="Score Range" prompt="Enter value between 1 and 5" sqref="C25:E28" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="Range error" error="Value not between 1 and 5" promptTitle="Score Range" prompt="Enter value between 1 and 5" sqref="C20:E26" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>0</formula1>
       <formula2>10</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="B22" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
-    <hyperlink ref="B8" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
-    <hyperlink ref="B9" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
-    <hyperlink ref="B23" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
+    <hyperlink ref="B17" r:id="rId1" display="Part 2 - Poster Presentation (guidelines) - 30%" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="B3" r:id="rId2" display="Part 1 - Written Report (guidelines) - 70%" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
+    <hyperlink ref="B18" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
   </hyperlinks>
   <printOptions gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3009,29 +3064,29 @@
   <sheetData>
     <row r="1" spans="1:2" ht="23" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="B5" s="2"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="36" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="38" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -3039,74 +3094,74 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="33" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="B12" s="47"/>
     </row>
     <row r="13" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="B13" s="47"/>
     </row>
     <row r="14" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="B14" s="47"/>
     </row>
     <row r="15" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="B15" s="47"/>
     </row>
     <row r="16" spans="1:2" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="B16" s="47"/>
     </row>
     <row r="17" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="B17" s="47"/>
     </row>
     <row r="18" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="39" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="B18" s="47"/>
     </row>
     <row r="19" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="39" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="B19" s="47"/>
     </row>
     <row r="20" spans="1:2" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="39" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="B20" s="47"/>
     </row>
     <row r="21" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="39" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="B21" s="47"/>
     </row>
@@ -3121,7 +3176,7 @@
     </row>
     <row r="23" spans="1:2" ht="35" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A23" s="41" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="B23" s="42" t="e">
         <f>B22*5</f>
@@ -3160,7 +3215,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="54.42578125" customWidth="1"/>
@@ -3174,22 +3229,22 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="36" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="38" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -3197,118 +3252,106 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B12" s="47"/>
     </row>
     <row r="13" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>88</v>
+        <v>114</v>
       </c>
       <c r="B13" s="47"/>
     </row>
-    <row r="14" spans="1:2" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>89</v>
+        <v>112</v>
       </c>
       <c r="B14" s="47"/>
     </row>
     <row r="15" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="B15" s="47"/>
     </row>
     <row r="16" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>91</v>
-      </c>
-      <c r="B16" s="47"/>
-    </row>
-    <row r="17" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+      <c r="B16" s="80"/>
+    </row>
+    <row r="17" spans="1:2" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>92</v>
-      </c>
-      <c r="B17" s="47"/>
+        <v>84</v>
+      </c>
+      <c r="B17" s="80"/>
     </row>
     <row r="18" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="39" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="B18" s="47"/>
     </row>
     <row r="19" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="39" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="B19" s="47"/>
     </row>
-    <row r="20" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="39" t="s">
-        <v>95</v>
-      </c>
-      <c r="B20" s="47"/>
-    </row>
-    <row r="21" spans="1:2" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+        <v>113</v>
+      </c>
+      <c r="B20" s="80"/>
+    </row>
+    <row r="21" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="39" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="B21" s="47"/>
     </row>
     <row r="22" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="39" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B22" s="47"/>
     </row>
     <row r="23" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="39" t="s">
-        <v>98</v>
-      </c>
-      <c r="B23" s="47"/>
-    </row>
-    <row r="24" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="39" t="s">
-        <v>99</v>
-      </c>
-      <c r="B24" s="47"/>
-    </row>
-    <row r="25" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="12" t="s">
+      <c r="A23" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B25" s="8" t="e">
-        <f>SUM(B12:B24)/COUNT(B12:B24)</f>
+      <c r="B23" s="8" t="e">
+        <f>SUM(B12:B22)/COUNT(B12:B22)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="41" t="s">
-        <v>100</v>
-      </c>
-      <c r="B26" s="42" t="e">
-        <f>B25*5</f>
+    <row r="24" spans="1:2" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="41" t="s">
+        <v>88</v>
+      </c>
+      <c r="B24" s="42" t="e">
+        <f>B23*5</f>
         <v>#DIV/0!</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1" selectLockedCells="1"/>
   <phoneticPr fontId="9" type="noConversion"/>
-  <conditionalFormatting sqref="B12:B24">
-    <cfRule type="colorScale" priority="1">
+  <conditionalFormatting sqref="B12:B22">
+    <cfRule type="colorScale" priority="21">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -3320,7 +3363,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="decimal" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Score out of range" error="Score range: 0-1" promptTitle="Score Range" prompt="Range: 0 - 1" sqref="B12:B24" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="decimal" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Score out of range" error="Score range: 0-1" promptTitle="Score Range" prompt="Range: 0 - 1" sqref="B12:B22" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>

</xml_diff>